<commit_message>
melhoria na interface (Gemini), corregção da inversão B4 e B1 na rota
</commit_message>
<xml_diff>
--- a/casos_aprovados/caso_2025_02_15/input.xlsx
+++ b/casos_aprovados/caso_2025_02_15/input.xlsx
@@ -538,7 +538,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -571,7 +570,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -669,11 +667,15 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="9" t="n"/>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>07:10</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr"/>
       <c r="F12" s="12" t="n"/>
       <c r="G12" s="12" t="n"/>
       <c r="H12" s="13" t="n"/>
@@ -720,11 +722,15 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="9" t="n"/>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr"/>
       <c r="F15" s="12" t="n"/>
       <c r="G15" s="12" t="n"/>
       <c r="H15" s="13" t="n"/>
@@ -737,11 +743,15 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="9" t="n"/>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr"/>
       <c r="F16" s="12" t="n"/>
       <c r="G16" s="12" t="n"/>
       <c r="H16" s="13" t="n"/>
@@ -1023,7 +1033,6 @@
       <c r="D45" s="5" t="n"/>
       <c r="E45" s="5" t="n"/>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="B47" s="2" t="inlineStr">
         <is>

</xml_diff>